<commit_message>
Make the explanations readable
Amounts with thousands separators, quantities without trailing zeros and
client terms in words ('7.5 % discount' instead of 'discount_pct 7.5').
Workbook rebuilt.
</commit_message>
<xml_diff>
--- a/reports/fee_billing_exceptions.xlsx
+++ b/reports/fee_billing_exceptions.xlsx
@@ -1080,7 +1080,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Activity of 538901758.77 with no invoice line</t>
+          <t>Activity of 538,901,758.77 with no invoice line</t>
         </is>
       </c>
     </row>
@@ -1137,7 +1137,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Client terms in force (flat_rate 0.90) were not applied, the invoice is at standard rates</t>
+          <t>Client terms in force (flat rate of 0.9) were not applied, the invoice is at standard rates</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -1199,7 +1199,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Client terms in force (flat_rate 0.90) were not applied, the invoice is at standard rates</t>
+          <t>Client terms in force (flat rate of 0.9) were not applied, the invoice is at standard rates</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -1261,7 +1261,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10320, C10916), each banded on its own. Priced as one client the fee is 21625.69</t>
+          <t>Billed under 2 client records (C10320, C10916), each banded on its own. Priced as one client the fee is 21,625.69</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -1323,7 +1323,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10320, C10916), each banded on its own. Priced as one client the fee is 16496.35</t>
+          <t>Billed under 2 client records (C10320, C10916), each banded on its own. Priced as one client the fee is 16,496.35</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1385,7 +1385,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10320, C10916), each banded on its own. Priced as one client the fee is 12471.76</t>
+          <t>Billed under 2 client records (C10320, C10916), each banded on its own. Priced as one client the fee is 12,471.76</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1447,7 +1447,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10320, C10916), each banded on its own. Priced as one client the fee is 12258.90</t>
+          <t>Billed under 2 client records (C10320, C10916), each banded on its own. Priced as one client the fee is 12,258.90</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1509,7 +1509,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10412, C10928), each banded on its own. Priced as one client the fee is 13354.20</t>
+          <t>Billed under 2 client records (C10412, C10928), each banded on its own. Priced as one client the fee is 13,354.20</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1571,7 +1571,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10330, C10948), each banded on its own. Priced as one client the fee is 16335.60</t>
+          <t>Billed under 2 client records (C10330, C10948), each banded on its own. Priced as one client the fee is 16,335.60</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10330, C10948), each banded on its own. Priced as one client the fee is 9188.66</t>
+          <t>Billed under 2 client records (C10330, C10948), each banded on its own. Priced as one client the fee is 9,188.66</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1695,7 +1695,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10412, C10928), each banded on its own. Priced as one client the fee is 13285.20</t>
+          <t>Billed under 2 client records (C10412, C10928), each banded on its own. Priced as one client the fee is 13,285.20</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1757,7 +1757,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10330, C10948), each banded on its own. Priced as one client the fee is 8638.97</t>
+          <t>Billed under 2 client records (C10330, C10948), each banded on its own. Priced as one client the fee is 8,638.97</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1819,7 +1819,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10330, C10948), each banded on its own. Priced as one client the fee is 13600.60</t>
+          <t>Billed under 2 client records (C10330, C10948), each banded on its own. Priced as one client the fee is 13,600.60</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -1881,7 +1881,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10330, C10948), each banded on its own. Priced as one client the fee is 12041.40</t>
+          <t>Billed under 2 client records (C10330, C10948), each banded on its own. Priced as one client the fee is 12,041.40</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -1943,7 +1943,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10412, C10928), each banded on its own. Priced as one client the fee is 11970.00</t>
+          <t>Billed under 2 client records (C10412, C10928), each banded on its own. Priced as one client the fee is 11,970.00</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -2005,7 +2005,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10330, C10948), each banded on its own. Priced as one client the fee is 11779.20</t>
+          <t>Billed under 2 client records (C10330, C10948), each banded on its own. Priced as one client the fee is 11,779.20</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -2067,7 +2067,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10412, C10928), each banded on its own. Priced as one client the fee is 11632.20</t>
+          <t>Billed under 2 client records (C10412, C10928), each banded on its own. Priced as one client the fee is 11,632.20</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -2129,7 +2129,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10300, C10979), each banded on its own. Priced as one client the fee is 8083.56</t>
+          <t>Billed under 2 client records (C10300, C10979), each banded on its own. Priced as one client the fee is 8,083.56</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -2191,7 +2191,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10330, C10948), each banded on its own. Priced as one client the fee is 11467.00</t>
+          <t>Billed under 2 client records (C10330, C10948), each banded on its own. Priced as one client the fee is 11,467.00</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -2253,7 +2253,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10412, C10928), each banded on its own. Priced as one client the fee is 11460.40</t>
+          <t>Billed under 2 client records (C10412, C10928), each banded on its own. Priced as one client the fee is 11,460.40</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -2315,7 +2315,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10412, C10928), each banded on its own. Priced as one client the fee is 11116.20</t>
+          <t>Billed under 2 client records (C10412, C10928), each banded on its own. Priced as one client the fee is 11,116.20</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -2377,7 +2377,7 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>Client terms in force (flat_rate 0.90) were not applied, the invoice is at standard rates</t>
+          <t>Client terms in force (flat rate of 0.9) were not applied, the invoice is at standard rates</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -2439,7 +2439,7 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10300, C10979), each banded on its own. Priced as one client the fee is 7584.13</t>
+          <t>Billed under 2 client records (C10300, C10979), each banded on its own. Priced as one client the fee is 7,584.13</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -2501,7 +2501,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10412, C10928), each banded on its own. Priced as one client the fee is 10962.60</t>
+          <t>Billed under 2 client records (C10412, C10928), each banded on its own. Priced as one client the fee is 10,962.60</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -2563,7 +2563,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10330, C10948), each banded on its own. Priced as one client the fee is 10905.00</t>
+          <t>Billed under 2 client records (C10330, C10948), each banded on its own. Priced as one client the fee is 10,905.00</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -2625,7 +2625,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 7429.98</t>
+          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 7,429.98</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -2687,7 +2687,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10330, C10948), each banded on its own. Priced as one client the fee is 7354.90</t>
+          <t>Billed under 2 client records (C10330, C10948), each banded on its own. Priced as one client the fee is 7,354.90</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -2749,7 +2749,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10330, C10948), each banded on its own. Priced as one client the fee is 8863.05</t>
+          <t>Billed under 2 client records (C10330, C10948), each banded on its own. Priced as one client the fee is 8,863.05</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -2811,7 +2811,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 7526.40</t>
+          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 7,526.40</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -2873,7 +2873,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 6514.65</t>
+          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 6,514.65</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -2935,7 +2935,7 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 6208.75</t>
+          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 6,208.75</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
@@ -3121,7 +3121,7 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10320, C10916), each banded on its own. Priced as one client the fee is 5066.85</t>
+          <t>Billed under 2 client records (C10320, C10916), each banded on its own. Priced as one client the fee is 5,066.85</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
@@ -3183,7 +3183,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10330, C10948), each banded on its own. Priced as one client the fee is 8500.15</t>
+          <t>Billed under 2 client records (C10330, C10948), each banded on its own. Priced as one client the fee is 8,500.15</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -3245,7 +3245,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10330, C10948), each banded on its own. Priced as one client the fee is 7176.11</t>
+          <t>Billed under 2 client records (C10330, C10948), each banded on its own. Priced as one client the fee is 7,176.11</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -3307,7 +3307,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10330, C10948), each banded on its own. Priced as one client the fee is 10327.40</t>
+          <t>Billed under 2 client records (C10330, C10948), each banded on its own. Priced as one client the fee is 10,327.40</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -3369,7 +3369,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10412, C10928), each banded on its own. Priced as one client the fee is 9854.30</t>
+          <t>Billed under 2 client records (C10412, C10928), each banded on its own. Priced as one client the fee is 9,854.30</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -3431,7 +3431,7 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10330, C10948), each banded on its own. Priced as one client the fee is 9430.60</t>
+          <t>Billed under 2 client records (C10330, C10948), each banded on its own. Priced as one client the fee is 9,430.60</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
@@ -3493,7 +3493,7 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10412, C10928), each banded on its own. Priced as one client the fee is 9119.95</t>
+          <t>Billed under 2 client records (C10412, C10928), each banded on its own. Priced as one client the fee is 9,119.95</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
@@ -3555,7 +3555,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10330, C10948), each banded on its own. Priced as one client the fee is 9001.20</t>
+          <t>Billed under 2 client records (C10330, C10948), each banded on its own. Priced as one client the fee is 9,001.20</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -3617,7 +3617,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 7492.60</t>
+          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 7,492.60</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
@@ -3679,7 +3679,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 7460.30</t>
+          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 7,460.30</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -3741,7 +3741,7 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 6822.85</t>
+          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 6,822.85</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
@@ -3803,7 +3803,7 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 6485.60</t>
+          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 6,485.60</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
@@ -3865,7 +3865,7 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 7107.05</t>
+          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 7,107.05</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
@@ -3927,7 +3927,7 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10412, C10928), each banded on its own. Priced as one client the fee is 12280.00</t>
+          <t>Billed under 2 client records (C10412, C10928), each banded on its own. Priced as one client the fee is 12,280.00</t>
         </is>
       </c>
       <c r="N49" t="inlineStr">
@@ -3989,7 +3989,7 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 5993.10</t>
+          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 5,993.10</t>
         </is>
       </c>
       <c r="N50" t="inlineStr">
@@ -4046,7 +4046,7 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>Client terms in force (discount_pct 7.5) were not applied, the invoice is at standard rates</t>
+          <t>Client terms in force (7.5 % discount) were not applied, the invoice is at standard rates</t>
         </is>
       </c>
       <c r="N51" t="inlineStr">
@@ -4103,7 +4103,7 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>Charged with the client terms (discount_pct 7.5) that ended on 2025-08-31</t>
+          <t>Charged with the client terms (7.5 % discount) that ended on 2025-08-31</t>
         </is>
       </c>
       <c r="N52" t="inlineStr">
@@ -4165,7 +4165,7 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 5639.15</t>
+          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 5,639.15</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
@@ -4227,7 +4227,7 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 8532.45</t>
+          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 8,532.45</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
@@ -4289,7 +4289,7 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10320, C10916), each banded on its own. Priced as one client the fee is 4380.00</t>
+          <t>Billed under 2 client records (C10320, C10916), each banded on its own. Priced as one client the fee is 4,380.00</t>
         </is>
       </c>
       <c r="N55" t="inlineStr">
@@ -4351,7 +4351,7 @@
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10300, C10979), each banded on its own. Priced as one client the fee is 4655.50</t>
+          <t>Billed under 2 client records (C10300, C10979), each banded on its own. Priced as one client the fee is 4,655.50</t>
         </is>
       </c>
       <c r="N56" t="inlineStr">
@@ -4413,7 +4413,7 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 5175.03</t>
+          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 5,175.03</t>
         </is>
       </c>
       <c r="N57" t="inlineStr">
@@ -4475,7 +4475,7 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 5160.90</t>
+          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 5,160.90</t>
         </is>
       </c>
       <c r="N58" t="inlineStr">
@@ -4537,7 +4537,7 @@
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 5089.93</t>
+          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 5,089.93</t>
         </is>
       </c>
       <c r="N59" t="inlineStr">
@@ -4599,7 +4599,7 @@
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 5036.87</t>
+          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 5,036.87</t>
         </is>
       </c>
       <c r="N60" t="inlineStr">
@@ -4661,7 +4661,7 @@
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 5006.06</t>
+          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 5,006.06</t>
         </is>
       </c>
       <c r="N61" t="inlineStr">
@@ -4723,7 +4723,7 @@
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 4995.52</t>
+          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 4,995.52</t>
         </is>
       </c>
       <c r="N62" t="inlineStr">
@@ -4785,7 +4785,7 @@
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 4919.61</t>
+          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 4,919.61</t>
         </is>
       </c>
       <c r="N63" t="inlineStr">
@@ -4847,7 +4847,7 @@
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 4875.34</t>
+          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 4,875.34</t>
         </is>
       </c>
       <c r="N64" t="inlineStr">
@@ -4909,7 +4909,7 @@
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 4835.00</t>
+          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 4,835.00</t>
         </is>
       </c>
       <c r="N65" t="inlineStr">
@@ -4971,7 +4971,7 @@
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 4814.01</t>
+          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 4,814.01</t>
         </is>
       </c>
       <c r="N66" t="inlineStr">
@@ -5033,7 +5033,7 @@
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10330, C10948), each banded on its own. Priced as one client the fee is 6050.19</t>
+          <t>Billed under 2 client records (C10330, C10948), each banded on its own. Priced as one client the fee is 6,050.19</t>
         </is>
       </c>
       <c r="N67" t="inlineStr">
@@ -5095,7 +5095,7 @@
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10330, C10948), each banded on its own. Priced as one client the fee is 6668.28</t>
+          <t>Billed under 2 client records (C10330, C10948), each banded on its own. Priced as one client the fee is 6,668.28</t>
         </is>
       </c>
       <c r="N68" t="inlineStr">
@@ -5157,7 +5157,7 @@
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10300, C10979), each banded on its own. Priced as one client the fee is 5246.22</t>
+          <t>Billed under 2 client records (C10300, C10979), each banded on its own. Priced as one client the fee is 5,246.22</t>
         </is>
       </c>
       <c r="N69" t="inlineStr">
@@ -5219,7 +5219,7 @@
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 4928.66</t>
+          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 4,928.66</t>
         </is>
       </c>
       <c r="N70" t="inlineStr">
@@ -5281,7 +5281,7 @@
       </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10300, C10979), each banded on its own. Priced as one client the fee is 4190.23</t>
+          <t>Billed under 2 client records (C10300, C10979), each banded on its own. Priced as one client the fee is 4,190.23</t>
         </is>
       </c>
       <c r="N71" t="inlineStr">
@@ -5343,7 +5343,7 @@
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 4108.60</t>
+          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 4,108.60</t>
         </is>
       </c>
       <c r="N72" t="inlineStr">
@@ -5405,7 +5405,7 @@
       </c>
       <c r="M73" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10300, C10979), each banded on its own. Priced as one client the fee is 3875.65</t>
+          <t>Billed under 2 client records (C10300, C10979), each banded on its own. Priced as one client the fee is 3,875.65</t>
         </is>
       </c>
       <c r="N73" t="inlineStr">
@@ -5591,7 +5591,7 @@
       </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 3929.43</t>
+          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 3,929.43</t>
         </is>
       </c>
       <c r="N76" t="inlineStr">
@@ -5653,7 +5653,7 @@
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 4704.87</t>
+          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 4,704.87</t>
         </is>
       </c>
       <c r="N77" t="inlineStr">
@@ -5715,7 +5715,7 @@
       </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 5491.50</t>
+          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 5,491.50</t>
         </is>
       </c>
       <c r="N78" t="inlineStr">
@@ -5777,7 +5777,7 @@
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 4653.08</t>
+          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 4,653.08</t>
         </is>
       </c>
       <c r="N79" t="inlineStr">
@@ -5839,7 +5839,7 @@
       </c>
       <c r="M80" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10330, C10948), each banded on its own. Priced as one client the fee is 10025.30</t>
+          <t>Billed under 2 client records (C10330, C10948), each banded on its own. Priced as one client the fee is 10,025.30</t>
         </is>
       </c>
       <c r="N80" t="inlineStr">
@@ -5901,7 +5901,7 @@
       </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10300, C10979), each banded on its own. Priced as one client the fee is 3975.31</t>
+          <t>Billed under 2 client records (C10300, C10979), each banded on its own. Priced as one client the fee is 3,975.31</t>
         </is>
       </c>
       <c r="N81" t="inlineStr">
@@ -5963,7 +5963,7 @@
       </c>
       <c r="M82" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10300, C10979), each banded on its own. Priced as one client the fee is 4536.75</t>
+          <t>Billed under 2 client records (C10300, C10979), each banded on its own. Priced as one client the fee is 4,536.75</t>
         </is>
       </c>
       <c r="N82" t="inlineStr">
@@ -6025,7 +6025,7 @@
       </c>
       <c r="M83" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10320, C10916), each banded on its own. Priced as one client the fee is 3995.65</t>
+          <t>Billed under 2 client records (C10320, C10916), each banded on its own. Priced as one client the fee is 3,995.65</t>
         </is>
       </c>
       <c r="N83" t="inlineStr">
@@ -6087,7 +6087,7 @@
       </c>
       <c r="M84" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10412, C10928), each banded on its own. Priced as one client the fee is 10437.60</t>
+          <t>Billed under 2 client records (C10412, C10928), each banded on its own. Priced as one client the fee is 10,437.60</t>
         </is>
       </c>
       <c r="N84" t="inlineStr">
@@ -6149,7 +6149,7 @@
       </c>
       <c r="M85" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10320, C10916), each banded on its own. Priced as one client the fee is 3926.85</t>
+          <t>Billed under 2 client records (C10320, C10916), each banded on its own. Priced as one client the fee is 3,926.85</t>
         </is>
       </c>
       <c r="N85" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="M86" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10320, C10916), each banded on its own. Priced as one client the fee is 3892.65</t>
+          <t>Billed under 2 client records (C10320, C10916), each banded on its own. Priced as one client the fee is 3,892.65</t>
         </is>
       </c>
       <c r="N86" t="inlineStr">
@@ -6325,7 +6325,7 @@
       </c>
       <c r="M88" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10300, C10979), each banded on its own. Priced as one client the fee is 3887.35</t>
+          <t>Billed under 2 client records (C10300, C10979), each banded on its own. Priced as one client the fee is 3,887.35</t>
         </is>
       </c>
       <c r="N88" t="inlineStr">
@@ -6387,7 +6387,7 @@
       </c>
       <c r="M89" t="inlineStr">
         <is>
-          <t>Invoice quantity 4283, activity 4938. The amount is right for the invoiced quantity</t>
+          <t>Invoice quantity 4,283, activity 4,938. The amount is right for the invoiced quantity</t>
         </is>
       </c>
       <c r="N89" t="inlineStr">
@@ -6449,7 +6449,7 @@
       </c>
       <c r="M90" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10300, C10979), each banded on its own. Priced as one client the fee is 3816.65</t>
+          <t>Billed under 2 client records (C10300, C10979), each banded on its own. Priced as one client the fee is 3,816.65</t>
         </is>
       </c>
       <c r="N90" t="inlineStr">
@@ -6511,7 +6511,7 @@
       </c>
       <c r="M91" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10300, C10979), each banded on its own. Priced as one client the fee is 3781.90</t>
+          <t>Billed under 2 client records (C10300, C10979), each banded on its own. Priced as one client the fee is 3,781.90</t>
         </is>
       </c>
       <c r="N91" t="inlineStr">
@@ -6573,7 +6573,7 @@
       </c>
       <c r="M92" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10300, C10979), each banded on its own. Priced as one client the fee is 3687.45</t>
+          <t>Billed under 2 client records (C10300, C10979), each banded on its own. Priced as one client the fee is 3,687.45</t>
         </is>
       </c>
       <c r="N92" t="inlineStr">
@@ -6635,7 +6635,7 @@
       </c>
       <c r="M93" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10320, C10916), each banded on its own. Priced as one client the fee is 3696.40</t>
+          <t>Billed under 2 client records (C10320, C10916), each banded on its own. Priced as one client the fee is 3,696.40</t>
         </is>
       </c>
       <c r="N93" t="inlineStr">
@@ -6697,7 +6697,7 @@
       </c>
       <c r="M94" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10300, C10979), each banded on its own. Priced as one client the fee is 4504.45</t>
+          <t>Billed under 2 client records (C10300, C10979), each banded on its own. Priced as one client the fee is 4,504.45</t>
         </is>
       </c>
       <c r="N94" t="inlineStr">
@@ -6759,7 +6759,7 @@
       </c>
       <c r="M95" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10055, C10941), each banded on its own. Priced as one client the fee is 3665.05</t>
+          <t>Billed under 2 client records (C10055, C10941), each banded on its own. Priced as one client the fee is 3,665.05</t>
         </is>
       </c>
       <c r="N95" t="inlineStr">
@@ -6821,7 +6821,7 @@
       </c>
       <c r="M96" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10055, C10941), each banded on its own. Priced as one client the fee is 3627.05</t>
+          <t>Billed under 2 client records (C10055, C10941), each banded on its own. Priced as one client the fee is 3,627.05</t>
         </is>
       </c>
       <c r="N96" t="inlineStr">
@@ -6883,7 +6883,7 @@
       </c>
       <c r="M97" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10320, C10916), each banded on its own. Priced as one client the fee is 3603.85</t>
+          <t>Billed under 2 client records (C10320, C10916), each banded on its own. Priced as one client the fee is 3,603.85</t>
         </is>
       </c>
       <c r="N97" t="inlineStr">
@@ -7059,7 +7059,7 @@
       </c>
       <c r="M100" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10320, C10916), each banded on its own. Priced as one client the fee is 3507.35</t>
+          <t>Billed under 2 client records (C10320, C10916), each banded on its own. Priced as one client the fee is 3,507.35</t>
         </is>
       </c>
       <c r="N100" t="inlineStr">
@@ -7121,7 +7121,7 @@
       </c>
       <c r="M101" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10300, C10979), each banded on its own. Priced as one client the fee is 3497.45</t>
+          <t>Billed under 2 client records (C10300, C10979), each banded on its own. Priced as one client the fee is 3,497.45</t>
         </is>
       </c>
       <c r="N101" t="inlineStr">
@@ -7245,7 +7245,7 @@
       </c>
       <c r="M103" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10300, C10979), each banded on its own. Priced as one client the fee is 3477.90</t>
+          <t>Billed under 2 client records (C10300, C10979), each banded on its own. Priced as one client the fee is 3,477.90</t>
         </is>
       </c>
       <c r="N103" t="inlineStr">
@@ -7307,7 +7307,7 @@
       </c>
       <c r="M104" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10300, C10979), each banded on its own. Priced as one client the fee is 3936.75</t>
+          <t>Billed under 2 client records (C10300, C10979), each banded on its own. Priced as one client the fee is 3,936.75</t>
         </is>
       </c>
       <c r="N104" t="inlineStr">
@@ -7369,7 +7369,7 @@
       </c>
       <c r="M105" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10320, C10916), each banded on its own. Priced as one client the fee is 4079.80</t>
+          <t>Billed under 2 client records (C10320, C10916), each banded on its own. Priced as one client the fee is 4,079.80</t>
         </is>
       </c>
       <c r="N105" t="inlineStr">
@@ -7431,7 +7431,7 @@
       </c>
       <c r="M106" t="inlineStr">
         <is>
-          <t>Charged with the client terms (discount_pct 10) that ended on 2025-06-30</t>
+          <t>Charged with the client terms (10 % discount) that ended on 2025-06-30</t>
         </is>
       </c>
       <c r="N106" t="inlineStr">
@@ -7493,7 +7493,7 @@
       </c>
       <c r="M107" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 4705.75</t>
+          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 4,705.75</t>
         </is>
       </c>
       <c r="N107" t="inlineStr">
@@ -7555,7 +7555,7 @@
       </c>
       <c r="M108" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10300, C10979), each banded on its own. Priced as one client the fee is 3838.90</t>
+          <t>Billed under 2 client records (C10300, C10979), each banded on its own. Priced as one client the fee is 3,838.90</t>
         </is>
       </c>
       <c r="N108" t="inlineStr">
@@ -7617,7 +7617,7 @@
       </c>
       <c r="M109" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10320, C10916), each banded on its own. Priced as one client the fee is 3301.20</t>
+          <t>Billed under 2 client records (C10320, C10916), each banded on its own. Priced as one client the fee is 3,301.20</t>
         </is>
       </c>
       <c r="N109" t="inlineStr">
@@ -7679,7 +7679,7 @@
       </c>
       <c r="M110" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10320, C10916), each banded on its own. Priced as one client the fee is 3284.10</t>
+          <t>Billed under 2 client records (C10320, C10916), each banded on its own. Priced as one client the fee is 3,284.10</t>
         </is>
       </c>
       <c r="N110" t="inlineStr">
@@ -7741,7 +7741,7 @@
       </c>
       <c r="M111" t="inlineStr">
         <is>
-          <t>Invoice quantity 5211, activity 4837. The amount is right for the invoiced quantity</t>
+          <t>Invoice quantity 5,211, activity 4,837. The amount is right for the invoiced quantity</t>
         </is>
       </c>
       <c r="N111" t="inlineStr">
@@ -7803,7 +7803,7 @@
       </c>
       <c r="M112" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10320, C10916), each banded on its own. Priced as one client the fee is 3212.85</t>
+          <t>Billed under 2 client records (C10320, C10916), each banded on its own. Priced as one client the fee is 3,212.85</t>
         </is>
       </c>
       <c r="N112" t="inlineStr">
@@ -7865,7 +7865,7 @@
       </c>
       <c r="M113" t="inlineStr">
         <is>
-          <t>Client terms in force (flat_rate 0.90) were not applied, the invoice is at standard rates</t>
+          <t>Client terms in force (flat rate of 0.9) were not applied, the invoice is at standard rates</t>
         </is>
       </c>
       <c r="N113" t="inlineStr">
@@ -7927,7 +7927,7 @@
       </c>
       <c r="M114" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10055, C10941), each banded on its own. Priced as one client the fee is 3112.15</t>
+          <t>Billed under 2 client records (C10055, C10941), each banded on its own. Priced as one client the fee is 3,112.15</t>
         </is>
       </c>
       <c r="N114" t="inlineStr">
@@ -8041,7 +8041,7 @@
       </c>
       <c r="M116" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10055, C10941), each banded on its own. Priced as one client the fee is 3149.75</t>
+          <t>Billed under 2 client records (C10055, C10941), each banded on its own. Priced as one client the fee is 3,149.75</t>
         </is>
       </c>
       <c r="N116" t="inlineStr">
@@ -8103,7 +8103,7 @@
       </c>
       <c r="M117" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 5521.35</t>
+          <t>Billed under 2 client records (C10311, C10969), each banded on its own. Priced as one client the fee is 5,521.35</t>
         </is>
       </c>
       <c r="N117" t="inlineStr">
@@ -8165,7 +8165,7 @@
       </c>
       <c r="M118" t="inlineStr">
         <is>
-          <t>Invoice quantity 5463, activity 6264. The amount is right for the invoiced quantity</t>
+          <t>Invoice quantity 5,463, activity 6,264. The amount is right for the invoiced quantity</t>
         </is>
       </c>
       <c r="N118" t="inlineStr">
@@ -8227,7 +8227,7 @@
       </c>
       <c r="M119" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10055, C10941), each banded on its own. Priced as one client the fee is 3120.30</t>
+          <t>Billed under 2 client records (C10055, C10941), each banded on its own. Priced as one client the fee is 3,120.30</t>
         </is>
       </c>
       <c r="N119" t="inlineStr">
@@ -8289,7 +8289,7 @@
       </c>
       <c r="M120" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10055, C10941), each banded on its own. Priced as one client the fee is 2961.80</t>
+          <t>Billed under 2 client records (C10055, C10941), each banded on its own. Priced as one client the fee is 2,961.80</t>
         </is>
       </c>
       <c r="N120" t="inlineStr">
@@ -8351,7 +8351,7 @@
       </c>
       <c r="M121" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10055, C10941), each banded on its own. Priced as one client the fee is 2844.20</t>
+          <t>Billed under 2 client records (C10055, C10941), each banded on its own. Priced as one client the fee is 2,844.20</t>
         </is>
       </c>
       <c r="N121" t="inlineStr">
@@ -8413,7 +8413,7 @@
       </c>
       <c r="M122" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10055, C10941), each banded on its own. Priced as one client the fee is 2548.80</t>
+          <t>Billed under 2 client records (C10055, C10941), each banded on its own. Priced as one client the fee is 2,548.80</t>
         </is>
       </c>
       <c r="N122" t="inlineStr">
@@ -8532,7 +8532,7 @@
       </c>
       <c r="M124" t="inlineStr">
         <is>
-          <t>Client terms in force (discount_pct 7.5) were not applied, the invoice is at standard rates</t>
+          <t>Client terms in force (7.5 % discount) were not applied, the invoice is at standard rates</t>
         </is>
       </c>
       <c r="N124" t="inlineStr">
@@ -8589,7 +8589,7 @@
       </c>
       <c r="M125" t="inlineStr">
         <is>
-          <t>Charged with the client terms (discount_pct 7.5) that ended on 2025-08-31</t>
+          <t>Charged with the client terms (7.5 % discount) that ended on 2025-08-31</t>
         </is>
       </c>
       <c r="N125" t="inlineStr">
@@ -8651,7 +8651,7 @@
       </c>
       <c r="M126" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10055, C10941), each banded on its own. Priced as one client the fee is 3109.30</t>
+          <t>Billed under 2 client records (C10055, C10941), each banded on its own. Priced as one client the fee is 3,109.30</t>
         </is>
       </c>
       <c r="N126" t="inlineStr">
@@ -8708,7 +8708,7 @@
       </c>
       <c r="M127" t="inlineStr">
         <is>
-          <t>Charged with the client terms (discount_pct 7.5) that ended on 2025-08-31</t>
+          <t>Charged with the client terms (7.5 % discount) that ended on 2025-08-31</t>
         </is>
       </c>
       <c r="N127" t="inlineStr">
@@ -8817,7 +8817,7 @@
       </c>
       <c r="M129" t="inlineStr">
         <is>
-          <t>Charged with the client terms (discount_pct 7.5) that ended on 2025-08-31</t>
+          <t>Charged with the client terms (7.5 % discount) that ended on 2025-08-31</t>
         </is>
       </c>
       <c r="N129" t="inlineStr">
@@ -8879,7 +8879,7 @@
       </c>
       <c r="M130" t="inlineStr">
         <is>
-          <t>Invoice quantity 4171, activity 4579. The amount is right for the invoiced quantity</t>
+          <t>Invoice quantity 4,171, activity 4,579. The amount is right for the invoiced quantity</t>
         </is>
       </c>
       <c r="N130" t="inlineStr">
@@ -8941,7 +8941,7 @@
       </c>
       <c r="M131" t="inlineStr">
         <is>
-          <t>Invoice quantity 5140, activity 4755. The amount is right for the invoiced quantity</t>
+          <t>Invoice quantity 5,140, activity 4,755. The amount is right for the invoiced quantity</t>
         </is>
       </c>
       <c r="N131" t="inlineStr">
@@ -9122,7 +9122,7 @@
       </c>
       <c r="M134" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10055, C10941), each banded on its own. Priced as one client the fee is 2651.00</t>
+          <t>Billed under 2 client records (C10055, C10941), each banded on its own. Priced as one client the fee is 2,651.00</t>
         </is>
       </c>
       <c r="N134" t="inlineStr">
@@ -9184,7 +9184,7 @@
       </c>
       <c r="M135" t="inlineStr">
         <is>
-          <t>Client terms in force (discount_pct 12.5) were not applied, the invoice is at standard rates</t>
+          <t>Client terms in force (12.5 % discount) were not applied, the invoice is at standard rates</t>
         </is>
       </c>
       <c r="N135" t="inlineStr">
@@ -9308,7 +9308,7 @@
       </c>
       <c r="M137" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10055, C10941), each banded on its own. Priced as one client the fee is 2467.35</t>
+          <t>Billed under 2 client records (C10055, C10941), each banded on its own. Priced as one client the fee is 2,467.35</t>
         </is>
       </c>
       <c r="N137" t="inlineStr">
@@ -9432,7 +9432,7 @@
       </c>
       <c r="M139" t="inlineStr">
         <is>
-          <t>Charged with the client terms (discount_pct 12.5) that ended on 2025-06-30</t>
+          <t>Charged with the client terms (12.5 % discount) that ended on 2025-06-30</t>
         </is>
       </c>
       <c r="N139" t="inlineStr">
@@ -9861,7 +9861,7 @@
       </c>
       <c r="M146" t="inlineStr">
         <is>
-          <t>Client terms in force (discount_pct 10) were not applied, the invoice is at standard rates</t>
+          <t>Client terms in force (10 % discount) were not applied, the invoice is at standard rates</t>
         </is>
       </c>
       <c r="N146" t="inlineStr">
@@ -9923,7 +9923,7 @@
       </c>
       <c r="M147" t="inlineStr">
         <is>
-          <t>Invoice quantity 1829, activity 2029. The amount is right for the invoiced quantity</t>
+          <t>Invoice quantity 1,829, activity 2,029. The amount is right for the invoiced quantity</t>
         </is>
       </c>
       <c r="N147" t="inlineStr">
@@ -9985,7 +9985,7 @@
       </c>
       <c r="M148" t="inlineStr">
         <is>
-          <t>Invoice quantity 2036, activity 2193. The amount is right for the invoiced quantity</t>
+          <t>Invoice quantity 2,036, activity 2,193. The amount is right for the invoiced quantity</t>
         </is>
       </c>
       <c r="N148" t="inlineStr">
@@ -10109,7 +10109,7 @@
       </c>
       <c r="M150" t="inlineStr">
         <is>
-          <t>Billed under 2 client records (C10055, C10941), each banded on its own. Priced as one client the fee is 2528.10</t>
+          <t>Billed under 2 client records (C10055, C10941), each banded on its own. Priced as one client the fee is 2,528.10</t>
         </is>
       </c>
       <c r="N150" t="inlineStr">
@@ -10409,7 +10409,7 @@
       </c>
       <c r="M155" t="inlineStr">
         <is>
-          <t>Charged with the client terms (discount_pct 12.5) that ended on 2025-06-30</t>
+          <t>Charged with the client terms (12.5 % discount) that ended on 2025-06-30</t>
         </is>
       </c>
       <c r="N155" t="inlineStr">
@@ -10471,7 +10471,7 @@
       </c>
       <c r="M156" t="inlineStr">
         <is>
-          <t>Charged with the client terms (discount_pct 12.5) that ended on 2025-06-30</t>
+          <t>Charged with the client terms (12.5 % discount) that ended on 2025-06-30</t>
         </is>
       </c>
       <c r="N156" t="inlineStr">

</xml_diff>